<commit_message>
Regenerate PDFs for the reworded sources
- Rockledge memo, risk assessment, and system inventory: rebuilt with
  LibreOffice, which reproduces the committed PDFs exactly from their prior
  sources (same pages, size, and text). The longer Annex III text overflowed
  three fixed row heights and was clipped in print, so those rows are taller
  in the two workbooks; cell contents are unchanged.
- Project 10 DPIA and the whitepaper: no build script exists for these, so
  they are rebuilt with pandoc and headless Chrome, styled to match the
  originals (DejaVu Sans A4 for the DPIA; Georgia/Helvetica/Menlo Letter for
  the whitepaper). Layout is close but not byte-identical: the whitepaper keeps
  10 pages and the DPIA runs 7 where the original ran 6, because the reworded
  text is longer. Drop this commit to keep the old PDFs and re-render them with
  the original pipeline instead.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05-rockledge-benefits-ai-governance/artifacts/ai_risk_assessment.xlsx
+++ b/05-rockledge-benefits-ai-governance/artifacts/ai_risk_assessment.xlsx
@@ -529,6 +529,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="35.05" customHeight="1" s="10">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -921,7 +922,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="79.84999999999999" customHeight="1" s="10">
+    <row r="8" ht="104" customHeight="1" s="10">
       <c r="A8" s="14" t="inlineStr">
         <is>
           <t>AIR-004</t>
@@ -1945,6 +1946,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="23.85" customHeight="1" s="10">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -2148,6 +2150,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="35.05" customHeight="1" s="10">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -2244,7 +2247,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="46.25" customHeight="1" s="10">
+    <row r="11" ht="64" customHeight="1" s="10">
       <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Contested classification</t>

</xml_diff>